<commit_message>
MAY BAN - 20/3
</commit_message>
<xml_diff>
--- a/.xlsx
+++ b/.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -444,7 +444,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>[D10_C1_B1_04]-M2. Tìm mệnh đề đúng (cảm thán, số là số gì, số chia hết cho, nghiệm của phương trình).</t>
+          <t>[D12_C4_B1_11]-M1. Tìm nguyên hàm của ax+b.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -454,10 +454,290 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>[D12_C4_B1_04]-M1. Tìm nguyên hàm asinx.</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>[D12_C4_B1_05]-M1. Tìm nguyên hàm acosx.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>[D12_C4_B1_28]-M1. Tìm nguyên hàm của m.e^x.</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>[D12_C4_B4_01]-M1. Cho F(a) và F(b). Tính t.phân từ a đến b.</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>[D12_C4_B4_04]-M2. Cho tích phân f. Tính t.phân (m.f+n).</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>TH</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>[D12_C4_B4_28]-M1. Tính t.phân a/cos^2x</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>[D12_C4_B4_29]-M1. Tính t.phân a/sin^2x</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>[D12_C4_B5_23]-M2. Tìm công thức tính diện tích từ hình vẽ có 2 parabol</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>[D12_C4_B5_24]-M2. Tìm công thức tính diện tích từ hình vẽ có đường thẳng và parabol</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>[D12_C4_B5_04]-M2. Diện tích hình phẳng: y=f(x),y=g(x)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>[D12_C5_B1_14]-M1. Cho PTMP, đọc véctơ pháp tuyến.</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>[D12_C5_B1_07]-M1. Tính khoảng cách từ điểm đến mặt phẳng.</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>[D12_C5_B1_01]-M2. Viết PTMP qua điểm và có véctơ pháp tuyến.</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>[D12_C5_B1_08]-M2. Xét vị trí giữa 2 mặt phẳng tùy ý.</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>